<commit_message>
Actividad #2 base de datos de academia
</commit_message>
<xml_diff>
--- a/Actividad #1/Formato diccionario de datos.xlsx
+++ b/Actividad #1/Formato diccionario de datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AdminSena\Documents\SENA2026\GRUPOS\ADSO3312932\Actividades\Desarrollar la Solución de Software\Construir la base de datos sql\SQL\Julio 24 de 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Analisis y desarrollo de software\Instructor Cesar Chacon\Cuarto Trimestre\Actividad #1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{129613F3-769C-40B9-AC90-01E1EDC1C026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3412C7-7CC5-49ED-ACB4-3669F0CAC948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{FA1876FA-84E8-4D3D-89B8-81A175F63CFA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FA1876FA-84E8-4D3D-89B8-81A175F63CFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,11 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
-  <si>
-    <t>DICCIONARIO DE DATOS PROYECTO
-XXXXXXXXXXX</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Descripción del Sistema de Información</t>
   </si>
@@ -72,10 +68,8 @@
     <t xml:space="preserve">Propiedades </t>
   </si>
   <si>
-    <t>Usuarios</t>
-  </si>
-  <si>
-    <t>IdUsuario</t>
+    <t>DICCIONARIO DE DATOS PROYECTO
+Academia</t>
   </si>
 </sst>
 </file>
@@ -347,17 +341,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -729,105 +723,105 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D05C5B2-DA1E-476D-9C9C-051B5ACABA31}">
   <dimension ref="B1:N54"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:14" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="19"/>
       <c r="C2" s="9"/>
-      <c r="D2" s="29" t="s">
-        <v>0</v>
+      <c r="D2" s="27" t="s">
+        <v>10</v>
       </c>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="20"/>
       <c r="C3" s="21"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D3" s="27"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D4" s="27"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-    </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D5" s="27"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="30"/>
-    </row>
-    <row r="7" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D6" s="27"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+    </row>
+    <row r="7" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="22"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-    </row>
-    <row r="8" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D7" s="27"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+    </row>
+    <row r="8" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -842,7 +836,7 @@
       <c r="M9" s="9"/>
       <c r="N9" s="10"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" s="23"/>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
@@ -857,7 +851,7 @@
       <c r="M10" s="21"/>
       <c r="N10" s="26"/>
     </row>
-    <row r="11" spans="2:14" ht="7.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:14" ht="7.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="6"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -872,9 +866,9 @@
       <c r="M11" s="11"/>
       <c r="N11" s="12"/>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -889,7 +883,7 @@
       <c r="M12" s="9"/>
       <c r="N12" s="10"/>
     </row>
-    <row r="13" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="6"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -904,9 +898,9 @@
       <c r="M13" s="11"/>
       <c r="N13" s="12"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -921,7 +915,7 @@
       <c r="M14" s="9"/>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -936,9 +930,9 @@
       <c r="M15" s="11"/>
       <c r="N15" s="12"/>
     </row>
-    <row r="16" spans="2:14" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
@@ -953,573 +947,569 @@
       <c r="M16" s="17"/>
       <c r="N16" s="18"/>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B18" s="28" t="s">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B18" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28" t="s">
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28" t="s">
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="1" t="s">
+      <c r="M18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="N18" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B19" s="27" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="29"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
+      <c r="K24" s="29"/>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="29"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
+      <c r="K27" s="29"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="27"/>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="29"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="29"/>
+      <c r="J30" s="29"/>
+      <c r="K30" s="29"/>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="27"/>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="29"/>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="27"/>
-      <c r="J32" s="27"/>
-      <c r="K32" s="27"/>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="27"/>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="29"/>
+      <c r="K33" s="29"/>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27"/>
-      <c r="J34" s="27"/>
-      <c r="K34" s="27"/>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="29"/>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="27"/>
-      <c r="J35" s="27"/>
-      <c r="K35" s="27"/>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B36" s="27"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="27"/>
-      <c r="I36" s="27"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="27"/>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="29"/>
+      <c r="K36" s="29"/>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
+      <c r="K37" s="29"/>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
-      <c r="K38" s="27"/>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="29"/>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="27"/>
-      <c r="K39" s="27"/>
+    <row r="39" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B39" s="29"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="29"/>
+      <c r="H39" s="29"/>
+      <c r="I39" s="29"/>
+      <c r="J39" s="29"/>
+      <c r="K39" s="29"/>
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="27"/>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="29"/>
+      <c r="K40" s="29"/>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B41" s="27"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
-      <c r="K41" s="27"/>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
+      <c r="I41" s="29"/>
+      <c r="J41" s="29"/>
+      <c r="K41" s="29"/>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
       <c r="N41" s="2"/>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B42" s="27"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="27"/>
-      <c r="J42" s="27"/>
-      <c r="K42" s="27"/>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="29"/>
+      <c r="J42" s="29"/>
+      <c r="K42" s="29"/>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B43" s="27"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="27"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27"/>
-      <c r="J43" s="27"/>
-      <c r="K43" s="27"/>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B44" s="27"/>
-      <c r="C44" s="27"/>
-      <c r="D44" s="27"/>
-      <c r="E44" s="27"/>
-      <c r="F44" s="27"/>
-      <c r="G44" s="27"/>
-      <c r="H44" s="27"/>
-      <c r="I44" s="27"/>
-      <c r="J44" s="27"/>
-      <c r="K44" s="27"/>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29"/>
+      <c r="H44" s="29"/>
+      <c r="I44" s="29"/>
+      <c r="J44" s="29"/>
+      <c r="K44" s="29"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B45" s="27"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="27"/>
-      <c r="E45" s="27"/>
-      <c r="F45" s="27"/>
-      <c r="G45" s="27"/>
-      <c r="H45" s="27"/>
-      <c r="I45" s="27"/>
-      <c r="J45" s="27"/>
-      <c r="K45" s="27"/>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B45" s="29"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="29"/>
+      <c r="H45" s="29"/>
+      <c r="I45" s="29"/>
+      <c r="J45" s="29"/>
+      <c r="K45" s="29"/>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B46" s="27"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="27"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="27"/>
-      <c r="H46" s="27"/>
-      <c r="I46" s="27"/>
-      <c r="J46" s="27"/>
-      <c r="K46" s="27"/>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+      <c r="J46" s="29"/>
+      <c r="K46" s="29"/>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
     </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B47" s="27"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="27"/>
-      <c r="E47" s="27"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="27"/>
-      <c r="J47" s="27"/>
-      <c r="K47" s="27"/>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+      <c r="H47" s="29"/>
+      <c r="I47" s="29"/>
+      <c r="J47" s="29"/>
+      <c r="K47" s="29"/>
       <c r="L47" s="2"/>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
     </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B48" s="27"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="27"/>
-      <c r="E48" s="27"/>
-      <c r="F48" s="27"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
-      <c r="I48" s="27"/>
-      <c r="J48" s="27"/>
-      <c r="K48" s="27"/>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="29"/>
+      <c r="J48" s="29"/>
+      <c r="K48" s="29"/>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
     </row>
-    <row r="49" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B49" s="27"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="27"/>
-      <c r="E49" s="27"/>
-      <c r="F49" s="27"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="27"/>
-      <c r="I49" s="27"/>
-      <c r="J49" s="27"/>
-      <c r="K49" s="27"/>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B49" s="29"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="29"/>
+      <c r="F49" s="29"/>
+      <c r="G49" s="29"/>
+      <c r="H49" s="29"/>
+      <c r="I49" s="29"/>
+      <c r="J49" s="29"/>
+      <c r="K49" s="29"/>
       <c r="L49" s="2"/>
       <c r="M49" s="2"/>
       <c r="N49" s="2"/>
     </row>
-    <row r="50" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B50" s="27"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="27"/>
-      <c r="E50" s="27"/>
-      <c r="F50" s="27"/>
-      <c r="G50" s="27"/>
-      <c r="H50" s="27"/>
-      <c r="I50" s="27"/>
-      <c r="J50" s="27"/>
-      <c r="K50" s="27"/>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="29"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="29"/>
+      <c r="H50" s="29"/>
+      <c r="I50" s="29"/>
+      <c r="J50" s="29"/>
+      <c r="K50" s="29"/>
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
       <c r="N50" s="2"/>
     </row>
-    <row r="51" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B51" s="27"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="27"/>
-      <c r="E51" s="27"/>
-      <c r="F51" s="27"/>
-      <c r="G51" s="27"/>
-      <c r="H51" s="27"/>
-      <c r="I51" s="27"/>
-      <c r="J51" s="27"/>
-      <c r="K51" s="27"/>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B51" s="29"/>
+      <c r="C51" s="29"/>
+      <c r="D51" s="29"/>
+      <c r="E51" s="29"/>
+      <c r="F51" s="29"/>
+      <c r="G51" s="29"/>
+      <c r="H51" s="29"/>
+      <c r="I51" s="29"/>
+      <c r="J51" s="29"/>
+      <c r="K51" s="29"/>
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
       <c r="N51" s="2"/>
     </row>
-    <row r="52" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B52" s="27"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
-      <c r="I52" s="27"/>
-      <c r="J52" s="27"/>
-      <c r="K52" s="27"/>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B52" s="29"/>
+      <c r="C52" s="29"/>
+      <c r="D52" s="29"/>
+      <c r="E52" s="29"/>
+      <c r="F52" s="29"/>
+      <c r="G52" s="29"/>
+      <c r="H52" s="29"/>
+      <c r="I52" s="29"/>
+      <c r="J52" s="29"/>
+      <c r="K52" s="29"/>
       <c r="L52" s="2"/>
       <c r="M52" s="2"/>
       <c r="N52" s="2"/>
     </row>
-    <row r="53" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B53" s="27"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="27"/>
-      <c r="E53" s="27"/>
-      <c r="F53" s="27"/>
-      <c r="G53" s="27"/>
-      <c r="H53" s="27"/>
-      <c r="I53" s="27"/>
-      <c r="J53" s="27"/>
-      <c r="K53" s="27"/>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B53" s="29"/>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
+      <c r="H53" s="29"/>
+      <c r="I53" s="29"/>
+      <c r="J53" s="29"/>
+      <c r="K53" s="29"/>
       <c r="L53" s="2"/>
       <c r="M53" s="2"/>
       <c r="N53" s="2"/>
     </row>
-    <row r="54" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B54" s="27"/>
-      <c r="C54" s="27"/>
-      <c r="D54" s="27"/>
-      <c r="E54" s="27"/>
-      <c r="F54" s="27"/>
-      <c r="G54" s="27"/>
-      <c r="H54" s="27"/>
-      <c r="I54" s="27"/>
-      <c r="J54" s="27"/>
-      <c r="K54" s="27"/>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B54" s="29"/>
+      <c r="C54" s="29"/>
+      <c r="D54" s="29"/>
+      <c r="E54" s="29"/>
+      <c r="F54" s="29"/>
+      <c r="G54" s="29"/>
+      <c r="H54" s="29"/>
+      <c r="I54" s="29"/>
+      <c r="J54" s="29"/>
+      <c r="K54" s="29"/>
       <c r="L54" s="2"/>
       <c r="M54" s="2"/>
       <c r="N54" s="2"/>

</xml_diff>